<commit_message>
Forms sync auto batch 3: 5000 files
</commit_message>
<xml_diff>
--- a/equipment_request_forms/040_technology_order_request_form--equipment_request_forms.xlsx
+++ b/equipment_request_forms/040_technology_order_request_form--equipment_request_forms.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -826,8 +826,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -855,12 +855,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{'value':_'laptop'}</t>
+          <t>laptop</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>{'value': 'Laptop'}</t>
+          <t>Laptop</t>
         </is>
       </c>
     </row>
@@ -872,12 +872,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'value':_'desktop'}</t>
+          <t>desktop</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>{'value': 'Desktop'}</t>
+          <t>Desktop</t>
         </is>
       </c>
     </row>
@@ -889,12 +889,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{'value':_'other'}</t>
+          <t>other</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>{'value': 'Other'}</t>
+          <t>Other</t>
         </is>
       </c>
     </row>

</xml_diff>